<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-02 Le rayon de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-02.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut chanter le refrain en classe. Le rayon d'or l'accompagne. Un chuchotement serre son ventre. Elle chante quand même. Le soir, elle raconte, puis elle reprend le refrain près de la fenêtre.</t>
+          <t>Mila veut parler maintenant. Un éclat de buée saute dans le rond de la vitre. Elle coupe papa : les mots se perdent. À l'école, une voix trop près serre le ventre ; elle coupe, trop vite. Elle refuse de foncer, attend à la table ronde, raconte. Merci vécu. L'éclat de buée tient le jaune.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon jaune s'étale sur les carreaux. Il touche le bord de la table ronde. De la buée couvre encore la vitre. Maman dessine un rond clair avec la main. Un oiseau passe tout près, tout vite. Le pain grille. Ça sent le beurre. Papa glisse une pomme dans la boîte. Tu as vu le petit rond dans la buée ? Oui. On voit le toit d'en face. Le soleil est là, même avec la buée. En ce moment, Mila souffle sur son lait. Une petite fumée danse au-dessus du bol. Doucement. Il est encore chaud. Il sent le matin, maman. À l'école, on chante aujourd'hui. Tu te souviens du refrain ? Un peu. Je veux le chanter avec la classe. Tu dis bonjour à la maîtresse. Oui. Bonjour, et merci. Mila pose le bol. Une goutte de lait reste sur la lèvre. Viens. J'essuie. Plus tard, l'école sent la craie et les cahiers. Le rayon entre aussi dans la classe. Il pose un carré d'or sur le tapis. Bonjour. On range les crayons, tout doux. Bonjour, maîtresse. Mila écoute. Elle pose son crayon bleu dans la boîte. Le bleu tape un tout petit coup. Merci, Mila. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près. Mila sent un malaise. Son ventre se serre. Elle pose les mains à plat sur la table. Elle reste assise. L'après-midi, la maîtresse parle encore. On chante tout doux. On écoute le refrain. Mila écoute encore. Elle chante avec la classe. Sa voix est petite. Son ventre est encore serré. Le soir, le rayon est parti de la cuisine. Il reste une lumière rose sur le mur. La porte s'ouvre. Te voilà. Tu as faim ? Mila pose son cartable. Elle regarde le mur rose. Le ventre est encore serré.</t>
+          <t>Les carreaux tiennent un bout de soleil. Le jaune glisse jusqu'à la table ronde. Sur la vitre, la buée fait un rideau blanc. Maman pose la paume au milieu du blanc. Un rond clair s'ouvre, minuscule. Dedans, un éclat de buée saute. Il brille, maman ! Tu le vois, toi ? Oui, dans le rond. Le toit d'en face passe par là. Ça sent le lait chaud, près du bol. Une fumée fine danse au-dessus. Une pomme rouge attend dans la boîte. Je veux dire quelque chose, maintenant ! On t'écoute après la pomme ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Le jaune, il marche sur les carreaux ! Les deux voix se cognent. Tu disais, Mila ? Le rayon. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le rond ? Parler. La boîte est prête. Mila glisse la pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Mila enfile la gauche, puis la droite. Au revoir, maman. Au revoir, Mila. Tu dis bonjour, là-bas ? Oui, papa. Un oiseau passe derrière le blanc. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Le rayon entre aussi dans la classe. Il pose un carré d'or sur le tapis. Bonjour. Bonjour, maîtresse. Mila s'assoit près du carré d'or. Le tapis est rêche sous ses genoux. Elle veut le dire, ce carré, maintenant. Une voix s'approche, trop près. La voix veut le tapis, elle aussi. Mila sent un malaise. Son ventre se serre, minuscule. Attends, je dois parler ! Ses mots se cognent à la voix. La voix part vers le tapis d'or. Mila referme la bouche. Les mains restent à plat sur ses genoux. Le soir, le rayon a quitté les carreaux. Il reste une lumière rose sur le mur. La porte s'ouvre. Te voilà, Mila. Tu as faim ? Mila pose le cartable près des chaussures. Le ventre est serré. Maman, j'ai un truc ! Maman range la boîte près de l'évier. Les mots de Mila tombent dans le bruit.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon jaune s'étale sur les carreaux. Il touche le bord de la table ronde. De la buée couvre encore la vitre. Maman dessine un rond clair avec la main. Un oiseau passe tout près, tout vite. Le pain grille. Ça sent le beurre. Papa glisse une pomme dans la boîte. Tu as vu le petit rond dans la buée ? Oui. On voit le toit d'en face. Le soleil est là, même avec la buée. En ce moment, Mila souffle sur son lait. Une petite fumée danse au-dessus du bol. Doucement. Il est encore chaud. Il sent le matin, maman. À l'école, on chante aujourd'hui. Tu te souviens du refrain ? Un peu. Je veux le chanter avec la classe. Tu dis bonjour à la maîtresse. Oui. Bonjour, et merci. Mila pose le bol. Une goutte de lait reste sur la lèvre. Viens. J'essuie. Plus tard, l'école sent la craie et les cahiers. Le rayon entre aussi dans la classe. Il pose un carré d'or sur le tapis. Bonjour. On range les crayons, tout doux. Bonjour, maîtresse. Mila écoute. Elle pose son crayon bleu dans la boîte. Le bleu tape un tout petit coup. Merci, Mila. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près. Mila sent un malaise. Son ventre se serre. Elle pose les mains à plat sur la table. Elle reste assise. L'après-midi, la maîtresse parle encore. On chante tout doux. On écoute le refrain. Mila écoute encore. Elle chante avec la classe. Sa voix est petite. Son ventre est encore serré. Le soir, le rayon est parti de la cuisine. Il reste une lumière rose sur le mur. La porte s'ouvre. Te voilà. Tu as faim ? Mila pose son cartable. Elle regarde le mur rose. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les carreaux tiennent un bout de soleil. Le jaune glisse jusqu'à la table ronde. Sur la vitre, la buée fait un rideau blanc. Maman pose la paume au milieu du blanc. Un rond clair s'ouvre, minuscule. Dedans, un &lt;emphasis level="moderate"&gt;éclat de buée&lt;/emphasis&gt; saute. Il brille, maman ! Tu le vois, toi ? Oui, dans le rond. Le toit d'en face passe par là. Ça sent le lait chaud, près du bol. Une fumée fine danse au-dessus. Une pomme rouge attend dans la boîte. Je veux dire quelque chose, maintenant ! On t'écoute après la pomme ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Le jaune, il marche sur les carreaux ! Les deux voix se cognent. Tu disais, Mila ? Le rayon. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le rond ? Parler. La boîte est prête. Mila glisse la pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Mila enfile la gauche, puis la droite. Au revoir, maman. Au revoir, Mila. Tu dis bonjour, là-bas ? Oui, papa. Un oiseau passe derrière le blanc. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Le rayon entre aussi dans la classe. Il pose un carré d'or sur le tapis. Bonjour. Bonjour, maîtresse. Mila s'assoit près du carré d'or. Le tapis est rêche sous ses genoux. Elle veut le dire, ce carré, maintenant. Une voix s'approche, trop près. La voix veut le tapis, elle aussi. Mila sent un malaise. Son ventre se serre, minuscule. Attends, je dois parler ! Ses mots se cognent à la voix. La voix part vers le tapis d'or. Mila referme la bouche. Les mains restent à plat sur ses genoux. Le soir, le rayon a quitté les carreaux. Il reste une lumière rose sur le mur. La porte s'ouvre. Te voilà, Mila. Tu as faim ? Mila pose le cartable près des chaussures. Le ventre est serré. Maman, j'ai un truc ! Maman range la boîte près de l'évier. Les mots de Mila tombent dans le bruit.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maya est à l'école. La maîtresse parle. Maya aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les crayons. Maya range son crayon. Elle écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Maya sent un malaise. Son ventre est serré. L'après-midi, la maîtresse parle encore. Elle dit : on chante tout doux. Maya écoute encore. Elle chante. Le soir, maman l'attend. Maya vient raconter à la maison. Elle dit : maman, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute. Maman dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. Maya dit : j'ai écouté le matin. J'ai écouté l'après-midi. Puis j'ai raconté. Maman serre sa main. Maya se sent plus légère. [pause]</t>
+          <t>Les carreaux tiennent un bout de soleil. Le jaune glisse jusqu'à la table ronde. Sur la vitre, la buée fait un rideau blanc. Maman pose la paume au milieu du blanc. Un rond clair s'ouvre, minuscule. Dedans, un &lt;emphasis&gt;éclat de buée&lt;/emphasis&gt; saute. Il brille, maman ! Tu le vois, toi ? Oui, dans le rond. Le toit d'en face passe par là. Ça sent le lait chaud, près du bol. Une fumée fine danse au-dessus. Une pomme rouge attend dans la boîte. Je veux dire quelque chose, maintenant ! On t'écoute après la pomme ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Le jaune, il marche sur les carreaux ! Les deux voix se cognent. Tu disais, Mila ? Le rayon. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le rond ? Parler. La boîte est prête. Mila glisse la pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Mila enfile la gauche, puis la droite. Au revoir, maman. Au revoir, Mila. Tu dis bonjour, là-bas ? Oui, papa. Un oiseau passe derrière le blanc. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Le rayon entre aussi dans la classe. Il pose un carré d'or sur le tapis. Bonjour. Bonjour, maîtresse. Mila s'assoit près du carré d'or. Le tapis est rêche sous ses genoux. Elle veut le dire, ce carré, maintenant. Une voix s'approche, trop près. La voix veut le tapis, elle aussi. Mila sent un malaise. Son ventre se serre, minuscule. Attends, je dois parler ! Ses mots se cognent à la voix. La voix part vers le tapis d'or. Mila referme la bouche. Les mains restent à plat sur ses genoux. Le soir, le rayon a quitté les carreaux. Il reste une lumière rose sur le mur. La porte s'ouvre. Te voilà, Mila. Tu as faim ? Mila pose le cartable près des chaussures. Le ventre est serré. Maman, j'ai un truc ! Maman range la boîte près de l'évier. Les mots de Mila tombent dans le bruit. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de buée</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,68 +1321,78 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=l_eclat_de_buee_dans_le_rond; tempo=naturel; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un rayon jaune s'étale sur les carreaux.
-narrateur|Il touche le bord de la table ronde.
-narrateur|De la buée couvre encore la vitre.
-narrateur|Maman dessine un rond clair avec la main.
-narrateur|Un oiseau passe tout près, tout vite.
-narrateur|Le pain grille.
-narrateur|Ça sent le beurre.
-narrateur|Papa glisse une pomme dans la boîte.
-maman|Tu as vu le petit rond dans la buée ?
-enfant-f|Oui.
-enfant-f|On voit le toit d'en face.
-papa|Le soleil est là, même avec la buée.
-narrateur|En ce moment, Mila souffle sur son lait.
-narrateur|Une petite fumée danse au-dessus du bol.
-maman|Doucement.
-maman|Il est encore chaud.
-enfant-f|Il sent le matin, maman.
-enfant-f|À l'école, on chante aujourd'hui.
-papa|Tu te souviens du refrain ?
-enfant-f|Un peu.
-enfant-f|Je veux le chanter avec la classe.
-maman|Tu dis bonjour à la maîtresse.
-enfant-f|Oui.
-enfant-f|Bonjour, et merci.
-narrateur|Mila pose le bol.
-narrateur|Une goutte de lait reste sur la lèvre.
-papa|Viens.
-papa|J'essuie.
-narrateur|Plus tard, l'école sent la craie et les cahiers.
+          <t>narrateur|Les carreaux tiennent un bout de soleil.
+narrateur|Le jaune glisse jusqu'à la table ronde.
+narrateur|Sur la vitre, la buée fait un rideau blanc.
+narrateur|Maman pose la paume au milieu du blanc.
+narrateur|Un rond clair s'ouvre, minuscule.
+narrateur|Dedans, un éclat de buée saute.
+enfant-f|Il brille, maman !
+maman|Tu le vois, toi ?
+enfant-f|Oui, dans le rond.
+papa|Le toit d'en face passe par là.
+narrateur|Ça sent le lait chaud, près du bol.
+narrateur|Une fumée fine danse au-dessus.
+narrateur|Une pomme rouge attend dans la boîte.
+enfant-f|Je veux dire quelque chose, maintenant !
+papa|On t'écoute après la pomme ?
+enfant-f|Maintenant !
+narrateur|En ce moment, Mila coupe la phrase de papa.
+enfant-f|Le jaune, il marche sur les carreaux !
+narrateur|Les deux voix se cognent.
+papa|Tu disais, Mila ?
+enfant-f|Le rayon.
+narrateur|Personne n'a la phrase entière.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux parler, ou regarder le rond ?
+enfant-f|Parler.
+maman|La boîte est prête.
+narrateur|Mila glisse la pomme dans la boîte.
+narrateur|Le cartable sent le cahier neuf.
+narrateur|Les chaussures attendent près de la porte.
+narrateur|Mila enfile la gauche, puis la droite.
+enfant-f|Au revoir, maman.
+maman|Au revoir, Mila.
+papa|Tu dis bonjour, là-bas ?
+enfant-f|Oui, papa.
+narrateur|Un oiseau passe derrière le blanc.
+narrateur|Plus tard, l'école sent la craie.
+narrateur|Les cahiers tapent un peu, dans le casier.
 narrateur|Le rayon entre aussi dans la classe.
 narrateur|Il pose un carré d'or sur le tapis.
 maitresse|Bonjour.
-maitresse|On range les crayons, tout doux.
 enfant-f|Bonjour, maîtresse.
-narrateur|Mila écoute.
-narrateur|Elle pose son crayon bleu dans la boîte.
-narrateur|Le bleu tape un tout petit coup.
-maitresse|Merci, Mila.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, tout près.
+narrateur|Mila s'assoit près du carré d'or.
+narrateur|Le tapis est rêche sous ses genoux.
+narrateur|Elle veut le dire, ce carré, maintenant.
+narrateur|Une voix s'approche, trop près.
+narrateur|La voix veut le tapis, elle aussi.
 narrateur|Mila sent un malaise.
-narrateur|Son ventre se serre.
-narrateur|Elle pose les mains à plat sur la table.
-narrateur|Elle reste assise.
-narrateur|L'après-midi, la maîtresse parle encore.
-maitresse|On chante tout doux.
-maitresse|On écoute le refrain.
-narrateur|Mila écoute encore.
-narrateur|Elle chante avec la classe.
-narrateur|Sa voix est petite.
-narrateur|Son ventre est encore serré.
-narrateur|Le soir, le rayon est parti de la cuisine.
+narrateur|Son ventre se serre, minuscule.
+enfant-f|Attends, je dois parler !
+narrateur|Ses mots se cognent à la voix.
+narrateur|La voix part vers le tapis d'or.
+narrateur|Mila referme la bouche.
+narrateur|Les mains restent à plat sur ses genoux.
+narrateur|Le soir, le rayon a quitté les carreaux.
 narrateur|Il reste une lumière rose sur le mur.
 narrateur|La porte s'ouvre.
-maman|Te voilà.
+maman|Te voilà, Mila.
 maman|Tu as faim ?
-narrateur|Mila pose son cartable.
-narrateur|Elle regarde le mur rose.
-narrateur|Le ventre est encore serré.</t>
+narrateur|Mila pose le cartable près des chaussures.
+narrateur|Le ventre est serré.
+enfant-f|Maman, j'ai un truc !
+narrateur|Maman range la boîte près de l'évier.
+narrateur|Les mots de Mila tombent dans le bruit.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1419,12 +1429,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila a un malaise. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Maya a un malaise. Que fait-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1434,7 +1444,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | elle raconte | à maman | à la maison | écouter</t>
+          <t>raconter | elle raconte | à maman | à la maison | écouter | elle attend | attendre | son tour</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1487,7 +1497,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,10 +1505,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1513,34 +1523,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1549,23 +1563,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_raconte_quand_le_silence_arrive; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1598,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret, tout bas. J'ai écouté le matin. J'ai écouté l'après-midi. Puis j'ai chanté, un peu. On t'écoute. Viens t'asseoir. Mila parle près de la tartine. Maman serre sa main. La main est tiède. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Mila se sent plus légère, comme le rayon.</t>
+          <t>Mila s'assoit à la table ronde. L'assiette claque un peu contre le bois. Maman, une voix a parlé ! Maman n'a pas fini de verser l'eau. L'eau est fraîche, Mila. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Dans sa poitrine, ça se bouscule. Mila refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. La tartine est pour toi. Papa pose l'assiette, sans se presser. On t'écoute, quand tu veux. Mila attend que le silence arrive. Sur la vitre, l'éclat de buée revient. Je peux dire quelque chose ? Oui, Mila. À l'école, une voix a parlé trop près. J'ai eu un malaise, dans le ventre. Je voulais le dire tout de suite. Les mots sont restés coincés. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret, tout bas. J'ai écouté le matin. J'ai écouté l'après-midi. Puis j'ai chanté, un peu. On t'écoute. Viens t'asseoir. Mila parle près de la tartine. Maman serre sa main. La main est tiède. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Mila se sent plus légère, comme le rayon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila s'assoit à la table ronde. L'assiette claque un peu contre le bois. Maman, une voix a parlé ! Maman n'a pas fini de verser l'eau. L'eau est fraîche, Mila. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Dans sa poitrine, ça se bouscule. Mila refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. La tartine est pour toi. Papa pose l'assiette, sans se presser. On t'écoute, quand tu veux. Mila attend que le silence arrive. Sur la vitre, l'&lt;emphasis level="moderate"&gt;éclat de buée&lt;/emphasis&gt; revient. Je peux dire quelque chose ? Oui, Mila. À l'école, une voix a parlé trop près. J'ai eu un malaise, dans le ventre. Je voulais le dire tout de suite. Les mots sont restés coincés. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Maya a écouté la maîtresse. Le matin, puis l'après-midi. Elle a raconté son malaise à la maison. [pause]</t>
+          <t>Mila s'assoit à la table ronde. L'assiette claque un peu contre le bois. Maman, une voix a parlé ! Maman n'a pas fini de verser l'eau. L'eau est fraîche, Mila. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Dans sa poitrine, ça se bouscule. Mila refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. La tartine est pour toi. Papa pose l'assiette, sans se presser. On t'écoute, quand tu veux. Mila attend que le silence arrive. Sur la vitre, l'&lt;emphasis&gt;éclat de buée&lt;/emphasis&gt; revient. Je peux dire quelque chose ? Oui, Mila. À l'école, une voix a parlé trop près. J'ai eu un malaise, dans le ventre. Je voulais le dire tout de suite. Les mots sont restés coincés. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1655,7 +1669,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1663,10 +1677,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1687,28 +1701,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>éclat de buée</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1735,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1733,26 +1751,48 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Maman.
-enfant-f|J'ai eu un malaise.
-enfant-f|Quelqu'un a parlé d'un secret, tout bas.
-enfant-f|J'ai écouté le matin.
-enfant-f|J'ai écouté l'après-midi.
-enfant-f|Puis j'ai chanté, un peu.
-maman|On t'écoute.
-papa|Viens t'asseoir.
-narrateur|Mila parle près de la tartine.
-narrateur|Maman serre sa main.
-narrateur|La main est tiède.
-maman|Tu as bien fait de raconter.
-papa|À l'école, on écoute la maîtresse.
-maman|Si tu as un malaise, tu viens le dire.
-narrateur|Mila se sent plus légère, comme le rayon.</t>
+          <t>narrateur|Mila s'assoit à la table ronde.
+narrateur|L'assiette claque un peu contre le bois.
+enfant-f|Maman, une voix a parlé !
+narrateur|Maman n'a pas fini de verser l'eau.
+maman|L'eau est fraîche, Mila.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute la cuisine, un instant.
+papa|La tartine est pour toi.
+narrateur|Papa pose l'assiette, sans se presser.
+maman|On t'écoute, quand tu veux.
+narrateur|Mila attend que le silence arrive.
+narrateur|Sur la vitre, l'éclat de buée revient.
+enfant-f|Je peux dire quelque chose ?
+papa|Oui, Mila.
+enfant-f|À l'école, une voix a parlé trop près.
+enfant-f|J'ai eu un malaise, dans le ventre.
+enfant-f|Je voulais le dire tout de suite.
+enfant-f|Les mots sont restés coincés.
+maman|Merci de nous le dire, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+papa|Tu as soif ?
+enfant-f|Un peu.
+narrateur|Mila prend une gorgée.
+narrateur|L'eau chante contre le verre.
+enfant-f|C'est frais.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>assiette,eau</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1819,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tu as fini ta tartine ? Oui. Merci, papa. Maman verse un verre d'eau. L'eau chante un peu contre le verre. Tu veux boire ? Oui, maman. Mila boit une gorgée. C'est frais. On reste encore un peu près de la fenêtre ? Oui. Le toit d'en face est rose. Mila chante le refrain, tout bas. Papa écoute. Maman écoute. Je le reconnais. C'est celui de la classe. La buée revient un peu. La cuisine est calme.</t>
+          <t>Mila glisse de la chaise. Le rond, je le montre ! Elle court vers la vitre. Elle essuie le blanc d'un grand geste. La buée part d'un coup. L'éclat de buée n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Son souffle revient sur le verre. Un petit blanc se reforme. Le jaune le traverse, sans bruit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de buée saute dans le rond. Il est revenu. Il m'a attendue. La table ronde garde la tartine.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Tu as fini ta tartine ? Oui. Merci, papa. Maman verse un verre d'eau. L'eau chante un peu contre le verre. Tu veux boire ? Oui, maman. Mila boit une gorgée. C'est frais. On reste encore un peu près de la fenêtre ? Oui. Le toit d'en face est rose. Mila chante le refrain, tout bas. Papa écoute. Maman écoute. Je le reconnais. C'est celui de la classe. La buée revient un peu. La cuisine est calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila glisse de la chaise. Le rond, je le montre ! Elle court vers la vitre. Elle essuie le blanc d'un grand geste. La buée part d'un coup. L'&lt;emphasis level="moderate"&gt;éclat de buée&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Son souffle revient sur le verre. Un petit blanc se reforme. Le jaune le traverse, sans bruit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de buée saute dans le rond. Il est revenu. Il m'a attendue. La table ronde garde la tartine.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maya boit un verre d'eau. Maman lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Mila glisse de la chaise. Le rond, je le montre ! Elle court vers la vitre. Elle essuie le blanc d'un grand geste. La buée part d'un coup. L'&lt;emphasis&gt;éclat de buée&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Son souffle revient sur le verre. Un petit blanc se reforme. Le jaune le traverse, sans bruit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de buée saute dans le rond. Il est revenu. Il m'a attendue. La table ronde garde la tartine.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1836,7 +1876,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1844,22 +1884,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1870,30 +1914,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de buée</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1902,42 +1946,55 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_buee; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|Tu as fini ta tartine ?
+          <t>narrateur|Mila glisse de la chaise.
+enfant-f|Le rond, je le montre !
+narrateur|Elle court vers la vitre.
+narrateur|Elle essuie le blanc d'un grand geste.
+narrateur|La buée part d'un coup.
+narrateur|L'éclat de buée n'est plus là.
+enfant-f|Il est parti !
+narrateur|Le sourire tremble.
+papa|Tu le cherches ?
 enfant-f|Oui.
-enfant-f|Merci, papa.
-narrateur|Maman verse un verre d'eau.
-narrateur|L'eau chante un peu contre le verre.
-maman|Tu veux boire ?
-enfant-f|Oui, maman.
-narrateur|Mila boit une gorgée.
-narrateur|C'est frais.
-papa|On reste encore un peu près de la fenêtre ?
-enfant-f|Oui.
-enfant-f|Le toit d'en face est rose.
-narrateur|Mila chante le refrain, tout bas.
-narrateur|Papa écoute.
-narrateur|Maman écoute.
-maman|Je le reconnais.
-enfant-f|C'est celui de la classe.
-narrateur|La buée revient un peu.
-narrateur|La cuisine est calme.</t>
+narrateur|Mila refuse de foncer.
+narrateur|Elle reste près de la vitre.
+narrateur|Personne ne parle.
+narrateur|Son souffle revient sur le verre.
+narrateur|Un petit blanc se reforme.
+narrateur|Le jaune le traverse, sans bruit.
+enfant-f|Comme ce matin !
+maman|Tu le vois, toi ?
+narrateur|Mila pose un doigt, sans frotter.
+narrateur|L'éclat de buée saute dans le rond.
+papa|Il est revenu.
+enfant-f|Il m'a attendue.
+narrateur|La table ronde garde la tartine.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>verre</t>
         </is>
       </c>
     </row>
@@ -1964,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le rayon a quitté les carreaux. Le toit d'en face reste rose. On t'a écoutée, Mila. Tu as chanté, puis tu as raconté.</t>
+          <t>La lumière rose tient sur le mur. On m'a entendue. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus chaud. Le toit d'en face est rose, lui aussi. Oui, papa. Le jaune repose dans le rond. Il est là. On le garde des yeux ? Oui. L'éclat de buée tient le jaune.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le rayon a quitté les carreaux. Le toit d'en face reste rose. On t'a écoutée, Mila. Tu as chanté, puis tu as raconté.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lumière rose tient sur le mur. On m'a entendue. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus chaud. Le toit d'en face est rose, lui aussi. Oui, papa. Le jaune repose dans le rond. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de buée&lt;/emphasis&gt; tient le jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lumière rose tient sur le mur. On m'a entendue. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus chaud. Le toit d'en face est rose, lui aussi. Oui, papa. Le jaune repose dans le rond. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis&gt;éclat de buée&lt;/emphasis&gt; tient le jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2021,7 +2078,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2029,10 +2086,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2041,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2055,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de buée</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2074,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2087,27 +2148,40 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_buee_tient_le_jaune; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le rayon a quitté les carreaux.
-narrateur|Le toit d'en face reste rose.
-papa|On t'a écoutée, Mila.
-maman|Tu as chanté, puis tu as raconté.</t>
+          <t>narrateur|La lumière rose tient sur le mur.
+enfant-f|On m'a entendue.
+maman|On reste un peu ?
+enfant-f|Oui, maman.
+narrateur|Mila serre le bol contre elle.
+narrateur|Le lait n'est plus chaud.
+papa|Le toit d'en face est rose, lui aussi.
+enfant-f|Oui, papa.
+narrateur|Le jaune repose dans le rond.
+enfant-f|Il est là.
+maman|On le garde des yeux ?
+enfant-f|Oui.
+narrateur|L'éclat de buée tient le jaune.</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2185,6 +2259,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>